<commit_message>
fix(firmware): blindaje v4 tras auditoria ronda 4 (GLM 5.3 y GPT Astra)
- caudalimetro.cpp: cambiar pinMode a INPUT (respeta pull-up 4.7k a 3.3V de Placa 2)
- config.h: acotar Q_MAX_FISICO_MLMIN a 2500 mL/min (filtro activo anti-ruido EMI) y clarificar tiempo de frenado
- darcy.h: corregir Rm nominal a 2.09e13 m^-1 segun ISO 8637 (K_UF especificado a 37 C)
- EN_USO_firmware_planta.ino: desactivar auto-calibracion ficticia de permeado; hacer qp opcional en calibracion bypass; silenciar datalogger al presionar STOP para eliminar muestras espurias
- PLANILLA_CALIBRACION_ENSAYOS_2_Y_3.xlsx: vaciar celdas sinteticas de entrada para registro experimental real
- AuditoriaIA: incluir dictamen de auditoria GLM 5.3 Flash
</commit_message>
<xml_diff>
--- a/02_Hito2_Instrumentacion_Sensores/02_Firmware_Test_Sensores/subhito2_2_v4/EN_USO_firmware_planta/PLANILLA_CALIBRACION_ENSAYOS_2_Y_3.xlsx
+++ b/02_Hito2_Instrumentacion_Sensores/02_Firmware_Test_Sensores/subhito2_2_v4/EN_USO_firmware_planta/PLANILLA_CALIBRACION_ENSAYOS_2_Y_3.xlsx
@@ -155,7 +155,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -191,11 +191,137 @@
         <color rgb="0022543D"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="0022543D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="0022543D"/>
+      </right>
+      <top style="medium">
+        <color rgb="0022543D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="0022543D"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="0022543D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="0022543D"/>
+      </right>
+      <top style="medium">
+        <color rgb="0022543D"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="0022543D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="0022543D"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="0022543D"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="0022543D"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="0022543D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="0022543D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="0022543D"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="0022543D"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -274,6 +400,14 @@
     <xf numFmtId="170" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -352,7 +486,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="13"/>
   <chart>
     <title>
       <tx>
@@ -475,7 +608,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="13"/>
   <chart>
     <title>
       <tx>
@@ -940,7 +1072,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -986,8 +1118,6 @@
           <t>Probeta Graduada de 1000 mL</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Manguera:</t>
@@ -998,10 +1128,6 @@
           <t>Silicona Flexible APM (Øint 12 mm, Øext 18 mm)</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
-      <c r="J5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1014,8 +1140,6 @@
           <t>Agua Desionizada / Limpia a 20 °C</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
       <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Cabezal:</t>
@@ -1026,10 +1150,6 @@
           <t>MBP-2000 (Rotor 3 rodillos a 120°)</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
-      <c r="J6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1042,8 +1162,6 @@
           <t>Leadshine DM860 (3200 pulsos/rev - 1/16 micropasos)</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Motor:</t>
@@ -1054,10 +1172,6 @@
           <t>Paso a Paso NEMA 34 (4.0 N·m)</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1070,8 +1184,6 @@
           <t>Owen Cañizares / Antonella Guitián / Enzo</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Ubicación:</t>
@@ -1082,10 +1194,6 @@
           <t>Laboratorio de Operaciones Unitarias - UNSa</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -1163,12 +1271,8 @@
       <c r="B12" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="12" t="n">
-        <v>272</v>
-      </c>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="12" t="n"/>
       <c r="E12" s="13">
         <f>IF(OR(D12="",C12=""),"",D12/C12)</f>
         <v/>
@@ -1201,12 +1305,8 @@
       <c r="B13" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="C13" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="12" t="n">
-        <v>408</v>
-      </c>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="12" t="n"/>
       <c r="E13" s="13">
         <f>IF(OR(D13="",C13=""),"",D13/C13)</f>
         <v/>
@@ -1239,12 +1339,8 @@
       <c r="B14" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="C14" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="12" t="n">
-        <v>544</v>
-      </c>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="12" t="n"/>
       <c r="E14" s="13">
         <f>IF(OR(D14="",C14=""),"",D14/C14)</f>
         <v/>
@@ -1277,12 +1373,8 @@
       <c r="B15" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="C15" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="12" t="n">
-        <v>680</v>
-      </c>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="12" t="n"/>
       <c r="E15" s="13">
         <f>IF(OR(D15="",C15=""),"",D15/C15)</f>
         <v/>
@@ -1315,12 +1407,8 @@
       <c r="B16" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>816</v>
-      </c>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="12" t="n"/>
       <c r="E16" s="13">
         <f>IF(OR(D16="",C16=""),"",D16/C16)</f>
         <v/>
@@ -1353,12 +1441,8 @@
       <c r="B17" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="C17" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="12" t="n">
-        <v>952</v>
-      </c>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="12" t="n"/>
       <c r="E17" s="13">
         <f>IF(OR(D17="",C17=""),"",D17/C17)</f>
         <v/>
@@ -1391,12 +1475,8 @@
       <c r="B18" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="C18" s="11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D18" s="12" t="n">
-        <v>544</v>
-      </c>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="12" t="n"/>
       <c r="E18" s="13">
         <f>IF(OR(D18="",C18=""),"",D18/C18)</f>
         <v/>
@@ -1429,12 +1509,8 @@
       <c r="B19" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="C19" s="11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D19" s="12" t="n">
-        <v>612</v>
-      </c>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="12" t="n"/>
       <c r="E19" s="13">
         <f>IF(OR(D19="",C19=""),"",D19/C19)</f>
         <v/>
@@ -1473,7 +1549,7 @@
           <t>Cilindrada Media (Promedio Aritmético):</t>
         </is>
       </c>
-      <c r="B22" s="20" t="n"/>
+      <c r="B22" s="34" t="n"/>
       <c r="C22" s="21">
         <f>AVERAGE(G12:G19)</f>
         <v/>
@@ -1493,7 +1569,7 @@
           <t>Desviación Estándar Muestral (σ):</t>
         </is>
       </c>
-      <c r="B23" s="20" t="n"/>
+      <c r="B23" s="34" t="n"/>
       <c r="C23" s="21">
         <f>STDEV.S(G12:G19)</f>
         <v/>
@@ -1513,7 +1589,7 @@
           <t>Coeficiente de Variación (CV%):</t>
         </is>
       </c>
-      <c r="B24" s="20" t="n"/>
+      <c r="B24" s="34" t="n"/>
       <c r="C24" s="23">
         <f>(C23/C22)*100</f>
         <v/>
@@ -1533,7 +1609,7 @@
           <t>Pendiente de Regresión Q vs RPM (Cilindrada):</t>
         </is>
       </c>
-      <c r="B25" s="20" t="n"/>
+      <c r="B25" s="34" t="n"/>
       <c r="C25" s="21">
         <f>SLOPE(E12:E19,B12:B19)</f>
         <v/>
@@ -1553,7 +1629,7 @@
           <t>Ordenada al Origen de Regresión (b):</t>
         </is>
       </c>
-      <c r="B26" s="20" t="n"/>
+      <c r="B26" s="34" t="n"/>
       <c r="C26" s="23">
         <f>INTERCEPT(E12:E19,B12:B19)</f>
         <v/>
@@ -1573,7 +1649,7 @@
           <t>Coeficiente de Determinación (R²):</t>
         </is>
       </c>
-      <c r="B27" s="20" t="n"/>
+      <c r="B27" s="34" t="n"/>
       <c r="C27" s="21">
         <f>RSQ(E12:E19,B12:B19)</f>
         <v/>
@@ -1593,12 +1669,12 @@
           <t>PARÁMETRO DEFINITIVO PARA EL FIRMWARE / SCADA</t>
         </is>
       </c>
-      <c r="B29" s="25" t="n"/>
-      <c r="C29" s="25" t="n"/>
-      <c r="D29" s="25" t="n"/>
-      <c r="E29" s="25" t="n"/>
-      <c r="F29" s="25" t="n"/>
-      <c r="G29" s="25" t="n"/>
+      <c r="B29" s="35" t="n"/>
+      <c r="C29" s="35" t="n"/>
+      <c r="D29" s="35" t="n"/>
+      <c r="E29" s="35" t="n"/>
+      <c r="F29" s="35" t="n"/>
+      <c r="G29" s="36" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="24" t="inlineStr">
@@ -1606,24 +1682,24 @@
           <t>Cilindrada Calibrada Bomba (ML_POR_VUELTA):</t>
         </is>
       </c>
-      <c r="B30" s="25" t="n"/>
-      <c r="C30" s="25" t="n"/>
-      <c r="D30" s="25" t="n"/>
-      <c r="E30" s="25" t="n"/>
+      <c r="B30" s="37" t="n"/>
+      <c r="C30" s="37" t="n"/>
+      <c r="D30" s="37" t="n"/>
+      <c r="E30" s="38" t="n"/>
       <c r="F30" s="26">
         <f>C25</f>
         <v/>
       </c>
-      <c r="G30" s="25" t="n"/>
+      <c r="G30" s="38" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="25" t="n"/>
-      <c r="B31" s="25" t="n"/>
-      <c r="C31" s="25" t="n"/>
-      <c r="D31" s="25" t="n"/>
-      <c r="E31" s="25" t="n"/>
-      <c r="F31" s="25" t="n"/>
-      <c r="G31" s="25" t="n"/>
+      <c r="A31" s="39" t="n"/>
+      <c r="B31" s="40" t="n"/>
+      <c r="C31" s="40" t="n"/>
+      <c r="D31" s="40" t="n"/>
+      <c r="E31" s="41" t="n"/>
+      <c r="F31" s="39" t="n"/>
+      <c r="G31" s="41" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
@@ -1631,12 +1707,12 @@
           <t>Ubicación en código: config.h -&gt; constexpr float ML_POR_VUELTA | En Web: Modo Desarrollador -&gt; Cilindrada Bomba</t>
         </is>
       </c>
-      <c r="B32" s="25" t="n"/>
-      <c r="C32" s="25" t="n"/>
-      <c r="D32" s="25" t="n"/>
-      <c r="E32" s="25" t="n"/>
-      <c r="F32" s="25" t="n"/>
-      <c r="G32" s="25" t="n"/>
+      <c r="B32" s="35" t="n"/>
+      <c r="C32" s="35" t="n"/>
+      <c r="D32" s="35" t="n"/>
+      <c r="E32" s="35" t="n"/>
+      <c r="F32" s="35" t="n"/>
+      <c r="G32" s="36" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="23">
@@ -1676,7 +1752,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -1724,9 +1800,6 @@
           <t>Efecto Hall YF-S401 (Impulsión / Alimentación)</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
       <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Pin ESP32:</t>
@@ -1737,11 +1810,6 @@
           <t>GPIO 14 (Borne 12 Superior)</t>
         </is>
       </c>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
-      <c r="J5" s="6" t="n"/>
-      <c r="K5" s="6" t="n"/>
-      <c r="L5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1754,9 +1822,6 @@
           <t>Filtro RC analógico (fc ≈ 338 Hz) + Blanking 1500 µs</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
       <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Probeta:</t>
@@ -1767,11 +1832,6 @@
           <t>Graduada de 1000 mL</t>
         </is>
       </c>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
-      <c r="J6" s="6" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1784,9 +1844,6 @@
           <t>98.00 Hz / (L/min) (5880.0 pulsos/L)</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
       <c r="F7" s="4" t="inlineStr">
         <is>
           <t>K Previo Owen:</t>
@@ -1797,11 +1854,6 @@
           <t>154.62 Hz / (L/min) (9277.2 pulsos/L)</t>
         </is>
       </c>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="n"/>
-      <c r="K7" s="6" t="n"/>
-      <c r="L7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1814,9 +1866,6 @@
           <t>Owen Cañizares / Antonella Guitián / Enzo</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
       <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Algoritmo:</t>
@@ -1827,11 +1876,6 @@
           <t>Período Recíproco con micros() en IRAM</t>
         </is>
       </c>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="n"/>
-      <c r="K8" s="6" t="n"/>
-      <c r="L8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -1921,15 +1965,9 @@
       <c r="B12" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="C12" s="28" t="n">
-        <v>42.06</v>
-      </c>
-      <c r="D12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="12" t="n">
-        <v>272</v>
-      </c>
+      <c r="C12" s="28" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="12" t="n"/>
       <c r="F12" s="13">
         <f>IF(OR(E12="",D12=""),"",E12/D12)</f>
         <v/>
@@ -1966,15 +2004,9 @@
       <c r="B13" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="C13" s="28" t="n">
-        <v>63.09</v>
-      </c>
-      <c r="D13" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="12" t="n">
-        <v>408</v>
-      </c>
+      <c r="C13" s="28" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="12" t="n"/>
       <c r="F13" s="13">
         <f>IF(OR(E13="",D13=""),"",E13/D13)</f>
         <v/>
@@ -2011,15 +2043,9 @@
       <c r="B14" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="C14" s="28" t="n">
-        <v>84.11</v>
-      </c>
-      <c r="D14" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="12" t="n">
-        <v>544</v>
-      </c>
+      <c r="C14" s="28" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="12" t="n"/>
       <c r="F14" s="13">
         <f>IF(OR(E14="",D14=""),"",E14/D14)</f>
         <v/>
@@ -2056,15 +2082,9 @@
       <c r="B15" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="C15" s="28" t="n">
-        <v>105.14</v>
-      </c>
-      <c r="D15" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="12" t="n">
-        <v>680</v>
-      </c>
+      <c r="C15" s="28" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="12" t="n"/>
       <c r="F15" s="13">
         <f>IF(OR(E15="",D15=""),"",E15/D15)</f>
         <v/>
@@ -2101,15 +2121,9 @@
       <c r="B16" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="C16" s="28" t="n">
-        <v>126.17</v>
-      </c>
-      <c r="D16" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="12" t="n">
-        <v>816</v>
-      </c>
+      <c r="C16" s="28" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="12" t="n"/>
       <c r="F16" s="13">
         <f>IF(OR(E16="",D16=""),"",E16/D16)</f>
         <v/>
@@ -2146,15 +2160,9 @@
       <c r="B17" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="C17" s="28" t="n">
-        <v>147.2</v>
-      </c>
-      <c r="D17" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="12" t="n">
-        <v>952</v>
-      </c>
+      <c r="C17" s="28" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="12" t="n"/>
       <c r="F17" s="13">
         <f>IF(OR(E17="",D17=""),"",E17/D17)</f>
         <v/>
@@ -2191,15 +2199,9 @@
       <c r="B18" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="C18" s="28" t="n">
-        <v>168.23</v>
-      </c>
-      <c r="D18" s="11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E18" s="12" t="n">
-        <v>544</v>
-      </c>
+      <c r="C18" s="28" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="12" t="n"/>
       <c r="F18" s="13">
         <f>IF(OR(E18="",D18=""),"",E18/D18)</f>
         <v/>
@@ -2236,15 +2238,9 @@
       <c r="B19" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="C19" s="28" t="n">
-        <v>189.26</v>
-      </c>
-      <c r="D19" s="11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E19" s="12" t="n">
-        <v>612</v>
-      </c>
+      <c r="C19" s="28" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="12" t="n"/>
       <c r="F19" s="13">
         <f>IF(OR(E19="",D19=""),"",E19/D19)</f>
         <v/>
@@ -2287,7 +2283,7 @@
           <t>Factor K Promedio (Media Aritmética):</t>
         </is>
       </c>
-      <c r="B22" s="20" t="n"/>
+      <c r="B22" s="34" t="n"/>
       <c r="C22" s="23">
         <f>AVERAGE(H12:H19)</f>
         <v/>
@@ -2307,7 +2303,7 @@
           <t>Desviación Estándar de K (σ):</t>
         </is>
       </c>
-      <c r="B23" s="20" t="n"/>
+      <c r="B23" s="34" t="n"/>
       <c r="C23" s="23">
         <f>STDEV.S(H12:H19)</f>
         <v/>
@@ -2327,7 +2323,7 @@
           <t>Coeficiente de Variación de K (CV%):</t>
         </is>
       </c>
-      <c r="B24" s="20" t="n"/>
+      <c r="B24" s="34" t="n"/>
       <c r="C24" s="23">
         <f>(C23/C22)*100</f>
         <v/>
@@ -2347,7 +2343,7 @@
           <t>Pulsos por Litro Promedio:</t>
         </is>
       </c>
-      <c r="B25" s="20" t="n"/>
+      <c r="B25" s="34" t="n"/>
       <c r="C25" s="30">
         <f>AVERAGE(I12:I19)</f>
         <v/>
@@ -2367,7 +2363,7 @@
           <t>Factor K por Regresión Lineal (Pendiente F vs Q [L/min]):</t>
         </is>
       </c>
-      <c r="B26" s="20" t="n"/>
+      <c r="B26" s="34" t="n"/>
       <c r="C26" s="23">
         <f>SLOPE(C12:C19,G12:G19)</f>
         <v/>
@@ -2387,7 +2383,7 @@
           <t>Ordenada al Origen de Regresión (Offset):</t>
         </is>
       </c>
-      <c r="B27" s="20" t="n"/>
+      <c r="B27" s="34" t="n"/>
       <c r="C27" s="23">
         <f>INTERCEPT(C12:C19,G12:G19)</f>
         <v/>
@@ -2407,7 +2403,7 @@
           <t>Coeficiente de Determinación (R²):</t>
         </is>
       </c>
-      <c r="B28" s="20" t="n"/>
+      <c r="B28" s="34" t="n"/>
       <c r="C28" s="21">
         <f>RSQ(C12:C19,G12:G19)</f>
         <v/>
@@ -2427,12 +2423,12 @@
           <t>PARÁMETROS DEFINITIVOS DE CALIBRACIÓN PARA EL FIRMWARE / SCADA</t>
         </is>
       </c>
-      <c r="B30" s="25" t="n"/>
-      <c r="C30" s="25" t="n"/>
-      <c r="D30" s="25" t="n"/>
-      <c r="E30" s="25" t="n"/>
-      <c r="F30" s="25" t="n"/>
-      <c r="G30" s="25" t="n"/>
+      <c r="B30" s="35" t="n"/>
+      <c r="C30" s="35" t="n"/>
+      <c r="D30" s="35" t="n"/>
+      <c r="E30" s="35" t="n"/>
+      <c r="F30" s="35" t="n"/>
+      <c r="G30" s="36" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="31" t="inlineStr">
@@ -2440,15 +2436,15 @@
           <t>Factor K Alimentación (K_ALIMENTACION):</t>
         </is>
       </c>
-      <c r="B31" s="25" t="n"/>
-      <c r="C31" s="25" t="n"/>
-      <c r="D31" s="25" t="n"/>
+      <c r="B31" s="35" t="n"/>
+      <c r="C31" s="35" t="n"/>
+      <c r="D31" s="36" t="n"/>
       <c r="E31" s="32">
         <f>C26</f>
         <v/>
       </c>
-      <c r="F31" s="25" t="n"/>
-      <c r="G31" s="25" t="n"/>
+      <c r="F31" s="35" t="n"/>
+      <c r="G31" s="36" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="31" t="inlineStr">
@@ -2456,15 +2452,15 @@
           <t>Equivalencia en Pulsos por Litro:</t>
         </is>
       </c>
-      <c r="B32" s="25" t="n"/>
-      <c r="C32" s="25" t="n"/>
-      <c r="D32" s="25" t="n"/>
+      <c r="B32" s="35" t="n"/>
+      <c r="C32" s="35" t="n"/>
+      <c r="D32" s="36" t="n"/>
       <c r="E32" s="33">
         <f>E31*60</f>
         <v/>
       </c>
-      <c r="F32" s="25" t="n"/>
-      <c r="G32" s="25" t="n"/>
+      <c r="F32" s="35" t="n"/>
+      <c r="G32" s="36" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
@@ -2472,12 +2468,12 @@
           <t>Ubicación en código: config.h -&gt; constexpr float K_ALIMENTACION | En Web: Modo Desarrollador -&gt; Factor K Alimentación</t>
         </is>
       </c>
-      <c r="B33" s="25" t="n"/>
-      <c r="C33" s="25" t="n"/>
-      <c r="D33" s="25" t="n"/>
-      <c r="E33" s="25" t="n"/>
-      <c r="F33" s="25" t="n"/>
-      <c r="G33" s="25" t="n"/>
+      <c r="B33" s="35" t="n"/>
+      <c r="C33" s="35" t="n"/>
+      <c r="D33" s="35" t="n"/>
+      <c r="E33" s="35" t="n"/>
+      <c r="F33" s="35" t="n"/>
+      <c r="G33" s="36" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="26">

</xml_diff>